<commit_message>
refatoração do código + llm
separação dos códigos em run_comparador, comparador e algoritmo (rapidfuzz, llm, elasticsearch)
</commit_message>
<xml_diff>
--- a/source/ago25/rapidfuzz/result_20250902_144805.xlsx
+++ b/source/ago25/rapidfuzz/result_20250902_144805.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\tcc-culturaeduca\source\ago25\rapidfuzz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A28659F-7CE7-471B-8FAA-20A098B6EB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D755A07-DF8A-4ABA-B272-E4D58A57693E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="7020" yWindow="1050" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enderecos" sheetId="1" r:id="rId1"/>
@@ -494,7 +494,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -504,6 +504,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -535,12 +541,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -850,6 +857,7 @@
   <cols>
     <col min="2" max="2" width="48.85546875" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="6" max="6" width="55.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1181,413 +1189,413 @@
         <v>106</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9">
+    <row r="9" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
         <v>4</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="3">
         <v>111</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="3">
         <v>70850</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="3">
         <v>111</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="3">
         <v>94.55</v>
       </c>
-      <c r="J9">
-        <v>100</v>
-      </c>
-      <c r="K9">
+      <c r="J9" s="3">
+        <v>100</v>
+      </c>
+      <c r="K9" s="3">
         <v>40</v>
       </c>
-      <c r="L9">
+      <c r="L9" s="3">
         <v>90.18</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="3" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10">
+    <row r="10" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
         <v>19</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="3">
         <v>635</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="3">
         <v>21410</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="3">
         <v>635</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="I10">
-        <v>100</v>
-      </c>
-      <c r="J10">
-        <v>100</v>
-      </c>
-      <c r="K10">
+      <c r="I10" s="3">
+        <v>100</v>
+      </c>
+      <c r="J10" s="3">
+        <v>100</v>
+      </c>
+      <c r="K10" s="3">
         <v>18.18</v>
       </c>
-      <c r="L10">
+      <c r="L10" s="3">
         <v>91.82</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M10" s="3" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11">
+    <row r="11" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
         <v>37</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="3">
         <v>635</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="3">
         <v>21410</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="3">
         <v>635</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="I11">
-        <v>100</v>
-      </c>
-      <c r="J11">
-        <v>100</v>
-      </c>
-      <c r="K11">
+      <c r="I11" s="3">
+        <v>100</v>
+      </c>
+      <c r="J11" s="3">
+        <v>100</v>
+      </c>
+      <c r="K11" s="3">
         <v>18.18</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="3">
         <v>91.82</v>
       </c>
-      <c r="M11" t="s">
+      <c r="M11" s="3" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12">
+    <row r="12" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
         <v>21</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="3">
         <v>129</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="3">
         <v>168293</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="3">
         <v>129</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="I12">
-        <v>100</v>
-      </c>
-      <c r="J12">
-        <v>100</v>
-      </c>
-      <c r="K12">
+      <c r="I12" s="3">
+        <v>100</v>
+      </c>
+      <c r="J12" s="3">
+        <v>100</v>
+      </c>
+      <c r="K12" s="3">
         <v>20</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="3">
         <v>92</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M12" s="3" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13">
+    <row r="13" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
         <v>13</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="3">
         <v>49</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="3">
         <v>69982</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="3">
         <v>49</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="I13">
-        <v>100</v>
-      </c>
-      <c r="J13">
-        <v>100</v>
-      </c>
-      <c r="K13">
+      <c r="I13" s="3">
+        <v>100</v>
+      </c>
+      <c r="J13" s="3">
+        <v>100</v>
+      </c>
+      <c r="K13" s="3">
         <v>23.53</v>
       </c>
-      <c r="L13">
+      <c r="L13" s="3">
         <v>92.35</v>
       </c>
-      <c r="M13" t="s">
+      <c r="M13" s="3" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14">
+    <row r="14" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
         <v>27</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="3">
         <v>290</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="3">
         <v>151049</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="3">
         <v>290</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="I14">
-        <v>100</v>
-      </c>
-      <c r="J14">
-        <v>100</v>
-      </c>
-      <c r="K14">
+      <c r="I14" s="3">
+        <v>100</v>
+      </c>
+      <c r="J14" s="3">
+        <v>100</v>
+      </c>
+      <c r="K14" s="3">
         <v>26.09</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="3">
         <v>92.61</v>
       </c>
-      <c r="M14" t="s">
+      <c r="M14" s="3" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15">
+    <row r="15" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
         <v>30</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="3">
         <v>605</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="3">
         <v>135351</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="3">
         <v>605</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="I15">
-        <v>100</v>
-      </c>
-      <c r="J15">
-        <v>100</v>
-      </c>
-      <c r="K15">
+      <c r="I15" s="3">
+        <v>100</v>
+      </c>
+      <c r="J15" s="3">
+        <v>100</v>
+      </c>
+      <c r="K15" s="3">
         <v>30</v>
       </c>
-      <c r="L15">
+      <c r="L15" s="3">
         <v>93</v>
       </c>
-      <c r="M15" t="s">
+      <c r="M15" s="3" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16">
+    <row r="16" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="3">
         <v>98</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="3">
         <v>15269</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="3">
         <v>98</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I16">
-        <v>100</v>
-      </c>
-      <c r="J16">
-        <v>100</v>
-      </c>
-      <c r="K16">
+      <c r="I16" s="3">
+        <v>100</v>
+      </c>
+      <c r="J16" s="3">
+        <v>100</v>
+      </c>
+      <c r="K16" s="3">
         <v>33.33</v>
       </c>
-      <c r="L16">
+      <c r="L16" s="3">
         <v>93.33</v>
       </c>
-      <c r="M16" t="s">
+      <c r="M16" s="3" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17">
+    <row r="17" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
         <v>35</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="3">
         <v>80</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="3">
         <v>82323</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="3">
         <v>80</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="I17">
-        <v>100</v>
-      </c>
-      <c r="J17">
-        <v>100</v>
-      </c>
-      <c r="K17">
+      <c r="I17" s="3">
+        <v>100</v>
+      </c>
+      <c r="J17" s="3">
+        <v>100</v>
+      </c>
+      <c r="K17" s="3">
         <v>35.29</v>
       </c>
-      <c r="L17">
+      <c r="L17" s="3">
         <v>93.53</v>
       </c>
-      <c r="M17" t="s">
+      <c r="M17" s="3" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18">
+    <row r="18" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
         <v>16</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="3">
         <v>679</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="3">
         <v>163095</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="3">
         <v>679</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="I18">
-        <v>100</v>
-      </c>
-      <c r="J18">
-        <v>100</v>
-      </c>
-      <c r="K18">
+      <c r="I18" s="3">
+        <v>100</v>
+      </c>
+      <c r="J18" s="3">
+        <v>100</v>
+      </c>
+      <c r="K18" s="3">
         <v>37.5</v>
       </c>
-      <c r="L18">
+      <c r="L18" s="3">
         <v>93.75</v>
       </c>
-      <c r="M18" t="s">
+      <c r="M18" s="3" t="s">
         <v>121</v>
       </c>
     </row>

</xml_diff>